<commit_message>
feat: Add migration preview test scripts and update generated Excel test data to adjust ZIS types.
</commit_message>
<xml_diff>
--- a/Backend/test_migration_files/testing_distribusi_excel.xlsx
+++ b/Backend/test_migration_files/testing_distribusi_excel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="151">
   <si>
     <t>Tanggal</t>
   </si>
@@ -127,196 +127,199 @@
     <t/>
   </si>
   <si>
+    <t>Zakat</t>
+  </si>
+  <si>
+    <t>Bantuan rutin 1</t>
+  </si>
+  <si>
+    <t>081111111111</t>
+  </si>
+  <si>
+    <t>diterima</t>
+  </si>
+  <si>
+    <t>06 Januari 2026</t>
+  </si>
+  <si>
+    <t>Bantuan Pengobatan Asnaf Miskin</t>
+  </si>
+  <si>
+    <t>Berobat</t>
+  </si>
+  <si>
+    <t>Tidak Rutin</t>
+  </si>
+  <si>
+    <t>222222</t>
+  </si>
+  <si>
+    <t>Siti Aminah</t>
+  </si>
+  <si>
+    <t>2171019988776655</t>
+  </si>
+  <si>
+    <t>Jl. Harapan Raya No 2</t>
+  </si>
+  <si>
+    <t>Belian</t>
+  </si>
+  <si>
+    <t>Batam Kota</t>
+  </si>
+  <si>
+    <t>Batam Sehat</t>
+  </si>
+  <si>
+    <t>Miskin</t>
+  </si>
+  <si>
+    <t>Bantuan RS</t>
+  </si>
+  <si>
+    <t>082222222222</t>
+  </si>
+  <si>
+    <t>07 Februari 2026</t>
+  </si>
+  <si>
+    <t>Bantuan Syiar Dakwah Asnaf Sabilillah</t>
+  </si>
+  <si>
+    <t>Sinergi Dakwah</t>
+  </si>
+  <si>
+    <t>333333</t>
+  </si>
+  <si>
+    <t>Rahmat Hidayat</t>
+  </si>
+  <si>
+    <t>2171013333333333</t>
+  </si>
+  <si>
+    <t>Jl. Sukajadi Asri 3</t>
+  </si>
+  <si>
+    <t>Sukajadi</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Batam Taqwa</t>
+  </si>
+  <si>
+    <t>Fisabillillah</t>
+  </si>
+  <si>
+    <t>Infak Tidak Terikat</t>
+  </si>
+  <si>
+    <t>Operasional Dakwah</t>
+  </si>
+  <si>
+    <t>083333333333</t>
+  </si>
+  <si>
+    <t>08 Februari 2026</t>
+  </si>
+  <si>
+    <t>Bantuan Pelunasan Utang Asnaf Gharimin</t>
+  </si>
+  <si>
+    <t>Pembayaran Hutang</t>
+  </si>
+  <si>
+    <t>444444</t>
+  </si>
+  <si>
+    <t>Santi Kurnia</t>
+  </si>
+  <si>
+    <t>2171014444444444</t>
+  </si>
+  <si>
+    <t>Komp. Muka Kuning 4</t>
+  </si>
+  <si>
+    <t>Muka Kuning</t>
+  </si>
+  <si>
+    <t>Sei Beduk</t>
+  </si>
+  <si>
+    <t>Gharimin</t>
+  </si>
+  <si>
+    <t>Pelunasan</t>
+  </si>
+  <si>
+    <t>084444444444</t>
+  </si>
+  <si>
+    <t>09 Maret 2026</t>
+  </si>
+  <si>
+    <t>Bantuan Biaya Hidup Asnaf Ibnu Sabil</t>
+  </si>
+  <si>
+    <t>B. Pemulangan Ibnusabil</t>
+  </si>
+  <si>
+    <t>555555</t>
+  </si>
+  <si>
+    <t>Bagus Ramadhan</t>
+  </si>
+  <si>
+    <t>2171015555555555</t>
+  </si>
+  <si>
+    <t>Jl. Tiban Asri 5</t>
+  </si>
+  <si>
+    <t>Tiban Lama</t>
+  </si>
+  <si>
+    <t>Sekupang</t>
+  </si>
+  <si>
+    <t>Ibnu Sabil</t>
+  </si>
+  <si>
+    <t>Tiket Pulang</t>
+  </si>
+  <si>
+    <t>085555555555</t>
+  </si>
+  <si>
+    <t>10 Maret 2026</t>
+  </si>
+  <si>
+    <t>Bantuan Penyaluran Fitrah Asnaf Fakir</t>
+  </si>
+  <si>
+    <t>Penyaluran Zakat Fitrah</t>
+  </si>
+  <si>
+    <t>666666</t>
+  </si>
+  <si>
+    <t>Joko Winarno</t>
+  </si>
+  <si>
+    <t>2171016666666666</t>
+  </si>
+  <si>
+    <t>Jl. Melati 6</t>
+  </si>
+  <si>
+    <t>Kampung Pelita</t>
+  </si>
+  <si>
     <t>Zakat Fitrah</t>
-  </si>
-  <si>
-    <t>Bantuan rutin 1</t>
-  </si>
-  <si>
-    <t>081111111111</t>
-  </si>
-  <si>
-    <t>diterima</t>
-  </si>
-  <si>
-    <t>06 Januari 2026</t>
-  </si>
-  <si>
-    <t>Bantuan Pengobatan Asnaf Miskin</t>
-  </si>
-  <si>
-    <t>Berobat</t>
-  </si>
-  <si>
-    <t>Tidak Rutin</t>
-  </si>
-  <si>
-    <t>222222</t>
-  </si>
-  <si>
-    <t>Siti Aminah</t>
-  </si>
-  <si>
-    <t>2171019988776655</t>
-  </si>
-  <si>
-    <t>Jl. Harapan Raya No 2</t>
-  </si>
-  <si>
-    <t>Belian</t>
-  </si>
-  <si>
-    <t>Batam Kota</t>
-  </si>
-  <si>
-    <t>Batam Sehat</t>
-  </si>
-  <si>
-    <t>Miskin</t>
-  </si>
-  <si>
-    <t>Bantuan RS</t>
-  </si>
-  <si>
-    <t>082222222222</t>
-  </si>
-  <si>
-    <t>07 Februari 2026</t>
-  </si>
-  <si>
-    <t>Bantuan Syiar Dakwah Asnaf Sabilillah</t>
-  </si>
-  <si>
-    <t>Sinergi Dakwah</t>
-  </si>
-  <si>
-    <t>333333</t>
-  </si>
-  <si>
-    <t>Rahmat Hidayat</t>
-  </si>
-  <si>
-    <t>2171013333333333</t>
-  </si>
-  <si>
-    <t>Jl. Sukajadi Asri 3</t>
-  </si>
-  <si>
-    <t>Sukajadi</t>
-  </si>
-  <si>
-    <t>Cash</t>
-  </si>
-  <si>
-    <t>Batam Taqwa</t>
-  </si>
-  <si>
-    <t>Fisabillillah</t>
-  </si>
-  <si>
-    <t>Infak Tidak Terikat</t>
-  </si>
-  <si>
-    <t>Operasional Dakwah</t>
-  </si>
-  <si>
-    <t>083333333333</t>
-  </si>
-  <si>
-    <t>08 Februari 2026</t>
-  </si>
-  <si>
-    <t>Bantuan Pelunasan Utang Asnaf Gharimin</t>
-  </si>
-  <si>
-    <t>Pembayaran Hutang</t>
-  </si>
-  <si>
-    <t>444444</t>
-  </si>
-  <si>
-    <t>Santi Kurnia</t>
-  </si>
-  <si>
-    <t>2171014444444444</t>
-  </si>
-  <si>
-    <t>Komp. Muka Kuning 4</t>
-  </si>
-  <si>
-    <t>Muka Kuning</t>
-  </si>
-  <si>
-    <t>Sei Beduk</t>
-  </si>
-  <si>
-    <t>Gharimin</t>
-  </si>
-  <si>
-    <t>Pelunasan</t>
-  </si>
-  <si>
-    <t>084444444444</t>
-  </si>
-  <si>
-    <t>09 Maret 2026</t>
-  </si>
-  <si>
-    <t>Bantuan Biaya Hidup Asnaf Ibnu Sabil</t>
-  </si>
-  <si>
-    <t>B. Pemulangan Ibnusabil</t>
-  </si>
-  <si>
-    <t>555555</t>
-  </si>
-  <si>
-    <t>Bagus Ramadhan</t>
-  </si>
-  <si>
-    <t>2171015555555555</t>
-  </si>
-  <si>
-    <t>Jl. Tiban Asri 5</t>
-  </si>
-  <si>
-    <t>Tiban Lama</t>
-  </si>
-  <si>
-    <t>Sekupang</t>
-  </si>
-  <si>
-    <t>Ibnu Sabil</t>
-  </si>
-  <si>
-    <t>Tiket Pulang</t>
-  </si>
-  <si>
-    <t>085555555555</t>
-  </si>
-  <si>
-    <t>10 Maret 2026</t>
-  </si>
-  <si>
-    <t>Bantuan Penyaluran Fitrah Asnaf Fakir</t>
-  </si>
-  <si>
-    <t>Penyaluran Zakat Fitrah</t>
-  </si>
-  <si>
-    <t>666666</t>
-  </si>
-  <si>
-    <t>Joko Winarno</t>
-  </si>
-  <si>
-    <t>2171016666666666</t>
-  </si>
-  <si>
-    <t>Jl. Melati 6</t>
-  </si>
-  <si>
-    <t>Kampung Pelita</t>
   </si>
   <si>
     <t>086666666666</t>
@@ -1325,10 +1328,10 @@
         <v>34</v>
       </c>
       <c r="T7" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
       <c r="U7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="V7" t="s">
         <v>37</v>
@@ -1339,34 +1342,34 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
         <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K8">
         <v>800000</v>
@@ -1378,7 +1381,7 @@
         <v>34</v>
       </c>
       <c r="N8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="O8" t="s">
         <v>53</v>
@@ -1396,10 +1399,10 @@
         <v>34</v>
       </c>
       <c r="T8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="U8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="V8" t="s">
         <v>37</v>
@@ -1410,34 +1413,34 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D9" t="s">
         <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K9">
         <v>150000</v>
@@ -1452,7 +1455,7 @@
         <v>65</v>
       </c>
       <c r="O9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P9" t="s">
         <v>37</v>
@@ -1467,10 +1470,10 @@
         <v>34</v>
       </c>
       <c r="T9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="U9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="V9" t="s">
         <v>37</v>
@@ -1481,28 +1484,28 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D10" t="s">
         <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I10" t="s">
         <v>50</v>
@@ -1517,10 +1520,10 @@
         <v>33</v>
       </c>
       <c r="M10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O10" t="s">
         <v>66</v>
@@ -1535,13 +1538,13 @@
         <v>38</v>
       </c>
       <c r="S10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="T10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="U10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="V10" t="s">
         <v>37</v>
@@ -1552,31 +1555,31 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D11" t="s">
         <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J11" t="s">
         <v>51</v>
@@ -1588,7 +1591,7 @@
         <v>33</v>
       </c>
       <c r="M11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="N11" t="s">
         <v>52</v>
@@ -1597,7 +1600,7 @@
         <v>66</v>
       </c>
       <c r="P11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Q11">
         <v>1</v>
@@ -1606,13 +1609,13 @@
         <v>38</v>
       </c>
       <c r="S11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="T11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="V11" t="s">
         <v>37</v>

</xml_diff>